<commit_message>
11/12: align readme deliverables and starter data/counts with the workbooks, and anchor retention citations and nist govern mappings in the notes. readme and starter files only.
</commit_message>
<xml_diff>
--- a/12_ai-governance-operating-model/exercises/starter/ai_governance_core.xlsx
+++ b/12_ai-governance-operating-model/exercises/starter/ai_governance_core.xlsx
@@ -1773,7 +1773,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Govern 6.2 — Mechanisms exist to communicate to relevant stakeholders the impacts of AI.</t>
+          <t>Govern 4.2 — Organizational teams document the risks and potential impacts of the AI technology they design, develop, deploy, evaluate, and use, and they communicate about the impacts more broadly.</t>
         </is>
       </c>
       <c r="C8" s="23" t="inlineStr">
@@ -2097,7 +2097,7 @@
       </c>
       <c r="B4" s="21" t="inlineStr">
         <is>
-          <t>NIST AI 100-1 Govern subcategory 6.1 = "Policies and procedures address AI risks from third-party entities." Govern 6.2 = "Contingency processes handle failures or incidents in third-party data or high-risk AI systems." Where the Govern Crosswalk maps internal reporting cadence to Govern 6.1 or stakeholder communication to Govern 6.2, the 6.x family's primary scope is third-party and contingency; broader stakeholder communication aligns with the Govern 5.x family ("Processes are in place for robust engagement with relevant AI actors") and reporting cadence within the organization aligns with Govern 1.x and 4.x. The 6.x mappings used here capture the third-party / external-vendor reporting view of those controls.</t>
+          <t>NIST AI 100-1 Govern subcategory 6.1 = "Policies and procedures address AI risks from third-party entities." Govern 6.2 = "Contingency processes handle failures or incidents in third-party data or high-risk AI systems." Where the Govern Crosswalk maps internal reporting cadence to Govern 6.1 or stakeholder communication to Govern 6.2, the 6.x family's primary scope is third-party and contingency; broader stakeholder communication aligns with the Govern 5.x family ("Processes are in place for robust engagement with relevant AI actors") and reporting cadence within the organization aligns with Govern 1.x and 4.x. Rows that concern third-party / external-vendor contingencies map to the 6.x family; the internal reporting-cadence row maps to Govern 4.2 (impact communication).</t>
         </is>
       </c>
     </row>

</xml_diff>